<commit_message>
Term-structure charts on a real time axis
The existing line charts put tenor labels on the category axis, so 1Y 2Y 3Y 5Y 7Y
10Y come out evenly spaced: the 5Y-10Y gap renders the same width as 1Y-2Y and
the curve shape is wrong. Four scatter charts now plot against tenor in years -
CDS market vs model, hazard and survival, default probability, and the SOFR zero
curve against T.

Needed a numeric years column for the x axis, taken from CDS_Quotes!B, since the
existing blocks only carried tenor labels.

Verified with the curve snapshot substituted for the external link: par 95.0000,
reprice 1.08e-05 bp, zero errors. Chart source ranges resolve - years 1/2/3/5/7/10,
market 40/55/70/95/115/135, model identical to two decimals, default probability
rising 0.0056 to 0.2126.

Model reproducing every quoted spread to two decimals is the strip closing on
itself, which is what the market-vs-model chart should show on demo data.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/CDS_Pricer.xlsx
+++ b/bloomberg/CDS_Pricer.xlsx
@@ -777,6 +777,125 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>SOFR zero curve</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Curves'!D5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Curves'!$B$6:$B$70</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Curves'!$D$6:$D$70</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>T (years)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>zero %</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
@@ -1429,6 +1548,434 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>CDS term structure - market vs model</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Curves'!B84</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Curves'!$F$85:$F$90</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Curves'!$B$85:$B$90</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Curves'!C84</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Curves'!$F$85:$F$90</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Curves'!$C$85:$C$90</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>tenor (years)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>spread (bp)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Hazard and survival term structure</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Curves'!B74</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Curves'!$E$75:$E$80</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Curves'!$B$75:$B$80</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Curves'!C74</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Curves'!$E$75:$E$80</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Curves'!$C$75:$C$80</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>tenor (years)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t/>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Default probability term structure</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Curves'!D74</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Curves'!$E$75:$E$80</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Curves'!$D$75:$D$80</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>tenor (years)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>1 - Q(t)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
@@ -1736,6 +2283,94 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>99</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="7" name="Chart 7"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>115</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="8" name="Chart 8"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId8"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>131</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="9" name="Chart 9"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>147</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="10" name="Chart 10"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId10"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -23809,7 +24444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E90"/>
+  <dimension ref="A1:F98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25059,6 +25694,11 @@
           <t>Default prob 1-Q</t>
         </is>
       </c>
+      <c r="E74" s="183" t="inlineStr">
+        <is>
+          <t>Years</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75">
@@ -25077,6 +25717,10 @@
         <f>Hazard_Bootstrap!F7</f>
         <v/>
       </c>
+      <c r="E75" s="32">
+        <f>CDS_Quotes!B7</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76">
@@ -25095,6 +25739,10 @@
         <f>Hazard_Bootstrap!F8</f>
         <v/>
       </c>
+      <c r="E76" s="32">
+        <f>CDS_Quotes!B8</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77">
@@ -25113,6 +25761,10 @@
         <f>Hazard_Bootstrap!F9</f>
         <v/>
       </c>
+      <c r="E77" s="32">
+        <f>CDS_Quotes!B9</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78">
@@ -25131,6 +25783,10 @@
         <f>Hazard_Bootstrap!F10</f>
         <v/>
       </c>
+      <c r="E78" s="32">
+        <f>CDS_Quotes!B10</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79">
@@ -25149,6 +25805,10 @@
         <f>Hazard_Bootstrap!F11</f>
         <v/>
       </c>
+      <c r="E79" s="32">
+        <f>CDS_Quotes!B11</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80">
@@ -25167,6 +25827,10 @@
         <f>Hazard_Bootstrap!F12</f>
         <v/>
       </c>
+      <c r="E80" s="32">
+        <f>CDS_Quotes!B12</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="67" t="inlineStr">
@@ -25199,6 +25863,11 @@
       <c r="E84" s="183" t="inlineStr">
         <is>
           <t>Traded spread</t>
+        </is>
+      </c>
+      <c r="F84" s="183" t="inlineStr">
+        <is>
+          <t>Years</t>
         </is>
       </c>
     </row>
@@ -25223,6 +25892,10 @@
         <f>CDS_Pricer!$B$15</f>
         <v/>
       </c>
+      <c r="F85" s="32">
+        <f>CDS_Quotes!B7</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86">
@@ -25245,6 +25918,10 @@
         <f>CDS_Pricer!$B$15</f>
         <v/>
       </c>
+      <c r="F86" s="32">
+        <f>CDS_Quotes!B8</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87">
@@ -25267,6 +25944,10 @@
         <f>CDS_Pricer!$B$15</f>
         <v/>
       </c>
+      <c r="F87" s="32">
+        <f>CDS_Quotes!B9</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88">
@@ -25289,6 +25970,10 @@
         <f>CDS_Pricer!$B$15</f>
         <v/>
       </c>
+      <c r="F88" s="32">
+        <f>CDS_Quotes!B10</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89">
@@ -25311,6 +25996,10 @@
         <f>CDS_Pricer!$B$15</f>
         <v/>
       </c>
+      <c r="F89" s="32">
+        <f>CDS_Quotes!B11</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90">
@@ -25332,6 +26021,17 @@
       <c r="E90" s="50">
         <f>CDS_Pricer!$B$15</f>
         <v/>
+      </c>
+      <c r="F90" s="32">
+        <f>CDS_Quotes!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="177" t="inlineStr">
+        <is>
+          <t>Term structure on a true time axis. The line charts above use tenor labels, which space 1Y-2Y and 5Y-10Y equally.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Empty CDSW capture must read blank, not zero
With CDS_Entities O:AC empty, INDEX returns 0 rather than blank, so the captured
column showed 0 and the Diff column echoed the model value. Eleven rows of
apparent differences that were just the model restated. N(...)=0 now reads as no
capture and both columns stay blank until something real is typed in.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/CDS_Pricer.xlsx
+++ b/bloomberg/CDS_Pricer.xlsx
@@ -13953,7 +13953,7 @@
     <row r="42">
       <c r="A42" s="177" t="inlineStr">
         <is>
-          <t>Blank until a CDSW capture is typed into CDS_Entities O:AC for the live name. Notional, coupon, maturity and traded spread there are context, not compared.</t>
+          <t>Blank until a CDSW capture is typed into CDS_Entities O:AC for the live name. A zero there reads as no capture, not as a captured zero.</t>
         </is>
       </c>
     </row>
@@ -13986,7 +13986,7 @@
         </is>
       </c>
       <c r="B44" s="87">
-        <f>IFERROR(INDEX(CDS_Entities!$S$5:$S$14,CDS_Parameters!$B$28),"")</f>
+        <f>IFERROR(IF(N(INDEX(CDS_Entities!$S$5:$S$14,CDS_Parameters!$B$28))=0,"",INDEX(CDS_Entities!$S$5:$S$14,CDS_Parameters!$B$28)),"")</f>
         <v/>
       </c>
       <c r="C44" s="93">
@@ -13994,7 +13994,7 @@
         <v/>
       </c>
       <c r="D44" s="93">
-        <f>IF(OR(B44="",NOT(ISNUMBER(B44))),"",C44-B44)</f>
+        <f>IF(OR(B44="",NOT(ISNUMBER(B44)),NOT(ISNUMBER(C44))),"",C44-B44)</f>
         <v/>
       </c>
     </row>
@@ -14005,7 +14005,7 @@
         </is>
       </c>
       <c r="B45" s="87">
-        <f>IFERROR(INDEX(CDS_Entities!$T$5:$T$14,CDS_Parameters!$B$28),"")</f>
+        <f>IFERROR(IF(N(INDEX(CDS_Entities!$T$5:$T$14,CDS_Parameters!$B$28))=0,"",INDEX(CDS_Entities!$T$5:$T$14,CDS_Parameters!$B$28)),"")</f>
         <v/>
       </c>
       <c r="C45" s="93">
@@ -14013,7 +14013,7 @@
         <v/>
       </c>
       <c r="D45" s="93">
-        <f>IF(OR(B45="",NOT(ISNUMBER(B45))),"",C45-B45)</f>
+        <f>IF(OR(B45="",NOT(ISNUMBER(B45)),NOT(ISNUMBER(C45))),"",C45-B45)</f>
         <v/>
       </c>
     </row>
@@ -14024,7 +14024,7 @@
         </is>
       </c>
       <c r="B46" s="87">
-        <f>IFERROR(INDEX(CDS_Entities!$U$5:$U$14,CDS_Parameters!$B$28),"")</f>
+        <f>IFERROR(IF(N(INDEX(CDS_Entities!$U$5:$U$14,CDS_Parameters!$B$28))=0,"",INDEX(CDS_Entities!$U$5:$U$14,CDS_Parameters!$B$28)),"")</f>
         <v/>
       </c>
       <c r="C46" s="93">
@@ -14032,7 +14032,7 @@
         <v/>
       </c>
       <c r="D46" s="93">
-        <f>IF(OR(B46="",NOT(ISNUMBER(B46))),"",C46-B46)</f>
+        <f>IF(OR(B46="",NOT(ISNUMBER(B46)),NOT(ISNUMBER(C46))),"",C46-B46)</f>
         <v/>
       </c>
     </row>
@@ -14043,7 +14043,7 @@
         </is>
       </c>
       <c r="B47" s="87">
-        <f>IFERROR(INDEX(CDS_Entities!$V$5:$V$14,CDS_Parameters!$B$28),"")</f>
+        <f>IFERROR(IF(N(INDEX(CDS_Entities!$V$5:$V$14,CDS_Parameters!$B$28))=0,"",INDEX(CDS_Entities!$V$5:$V$14,CDS_Parameters!$B$28)),"")</f>
         <v/>
       </c>
       <c r="C47" s="93">
@@ -14051,7 +14051,7 @@
         <v/>
       </c>
       <c r="D47" s="93">
-        <f>IF(OR(B47="",NOT(ISNUMBER(B47))),"",C47-B47)</f>
+        <f>IF(OR(B47="",NOT(ISNUMBER(B47)),NOT(ISNUMBER(C47))),"",C47-B47)</f>
         <v/>
       </c>
     </row>
@@ -14062,7 +14062,7 @@
         </is>
       </c>
       <c r="B48" s="87">
-        <f>IFERROR(INDEX(CDS_Entities!$W$5:$W$14,CDS_Parameters!$B$28),"")</f>
+        <f>IFERROR(IF(N(INDEX(CDS_Entities!$W$5:$W$14,CDS_Parameters!$B$28))=0,"",INDEX(CDS_Entities!$W$5:$W$14,CDS_Parameters!$B$28)),"")</f>
         <v/>
       </c>
       <c r="C48" s="93">
@@ -14070,7 +14070,7 @@
         <v/>
       </c>
       <c r="D48" s="93">
-        <f>IF(OR(B48="",NOT(ISNUMBER(B48))),"",C48-B48)</f>
+        <f>IF(OR(B48="",NOT(ISNUMBER(B48)),NOT(ISNUMBER(C48))),"",C48-B48)</f>
         <v/>
       </c>
     </row>
@@ -14081,7 +14081,7 @@
         </is>
       </c>
       <c r="B49" s="87">
-        <f>IFERROR(INDEX(CDS_Entities!$X$5:$X$14,CDS_Parameters!$B$28),"")</f>
+        <f>IFERROR(IF(N(INDEX(CDS_Entities!$X$5:$X$14,CDS_Parameters!$B$28))=0,"",INDEX(CDS_Entities!$X$5:$X$14,CDS_Parameters!$B$28)),"")</f>
         <v/>
       </c>
       <c r="C49" s="93">
@@ -14089,7 +14089,7 @@
         <v/>
       </c>
       <c r="D49" s="93">
-        <f>IF(OR(B49="",NOT(ISNUMBER(B49))),"",C49-B49)</f>
+        <f>IF(OR(B49="",NOT(ISNUMBER(B49)),NOT(ISNUMBER(C49))),"",C49-B49)</f>
         <v/>
       </c>
     </row>
@@ -14100,7 +14100,7 @@
         </is>
       </c>
       <c r="B50" s="87">
-        <f>IFERROR(INDEX(CDS_Entities!$AB$5:$AB$14,CDS_Parameters!$B$28),"")</f>
+        <f>IFERROR(IF(N(INDEX(CDS_Entities!$AB$5:$AB$14,CDS_Parameters!$B$28))=0,"",INDEX(CDS_Entities!$AB$5:$AB$14,CDS_Parameters!$B$28)),"")</f>
         <v/>
       </c>
       <c r="C50" s="93">
@@ -14108,7 +14108,7 @@
         <v/>
       </c>
       <c r="D50" s="93">
-        <f>IF(OR(B50="",NOT(ISNUMBER(B50))),"",C50-B50)</f>
+        <f>IF(OR(B50="",NOT(ISNUMBER(B50)),NOT(ISNUMBER(C50))),"",C50-B50)</f>
         <v/>
       </c>
     </row>
@@ -14119,7 +14119,7 @@
         </is>
       </c>
       <c r="B51" s="180">
-        <f>IFERROR(INDEX(CDS_Entities!$Y$5:$Y$14,CDS_Parameters!$B$28),"")</f>
+        <f>IFERROR(IF(N(INDEX(CDS_Entities!$Y$5:$Y$14,CDS_Parameters!$B$28))=0,"",INDEX(CDS_Entities!$Y$5:$Y$14,CDS_Parameters!$B$28)),"")</f>
         <v/>
       </c>
       <c r="C51" s="180">
@@ -14127,7 +14127,7 @@
         <v/>
       </c>
       <c r="D51" s="180">
-        <f>IF(OR(B51="",NOT(ISNUMBER(B51))),"",C51-B51)</f>
+        <f>IF(OR(B51="",NOT(ISNUMBER(B51)),NOT(ISNUMBER(C51))),"",C51-B51)</f>
         <v/>
       </c>
     </row>
@@ -14138,7 +14138,7 @@
         </is>
       </c>
       <c r="B52" s="180">
-        <f>IFERROR(INDEX(CDS_Entities!$Z$5:$Z$14,CDS_Parameters!$B$28),"")</f>
+        <f>IFERROR(IF(N(INDEX(CDS_Entities!$Z$5:$Z$14,CDS_Parameters!$B$28))=0,"",INDEX(CDS_Entities!$Z$5:$Z$14,CDS_Parameters!$B$28)),"")</f>
         <v/>
       </c>
       <c r="C52" s="180">
@@ -14146,7 +14146,7 @@
         <v/>
       </c>
       <c r="D52" s="180">
-        <f>IF(OR(B52="",NOT(ISNUMBER(B52))),"",C52-B52)</f>
+        <f>IF(OR(B52="",NOT(ISNUMBER(B52)),NOT(ISNUMBER(C52))),"",C52-B52)</f>
         <v/>
       </c>
     </row>
@@ -14157,7 +14157,7 @@
         </is>
       </c>
       <c r="B53" s="180">
-        <f>IFERROR(INDEX(CDS_Entities!$AA$5:$AA$14,CDS_Parameters!$B$28),"")</f>
+        <f>IFERROR(IF(N(INDEX(CDS_Entities!$AA$5:$AA$14,CDS_Parameters!$B$28))=0,"",INDEX(CDS_Entities!$AA$5:$AA$14,CDS_Parameters!$B$28)),"")</f>
         <v/>
       </c>
       <c r="C53" s="180">
@@ -14165,7 +14165,7 @@
         <v/>
       </c>
       <c r="D53" s="180">
-        <f>IF(OR(B53="",NOT(ISNUMBER(B53))),"",C53-B53)</f>
+        <f>IF(OR(B53="",NOT(ISNUMBER(B53)),NOT(ISNUMBER(C53))),"",C53-B53)</f>
         <v/>
       </c>
     </row>
@@ -14176,7 +14176,7 @@
         </is>
       </c>
       <c r="B54" s="180">
-        <f>IFERROR(INDEX(CDS_Entities!$AC$5:$AC$14,CDS_Parameters!$B$28),"")</f>
+        <f>IFERROR(IF(N(INDEX(CDS_Entities!$AC$5:$AC$14,CDS_Parameters!$B$28))=0,"",INDEX(CDS_Entities!$AC$5:$AC$14,CDS_Parameters!$B$28)),"")</f>
         <v/>
       </c>
       <c r="C54" s="180">

</xml_diff>

<commit_message>
Add a CDSRisk probe so a blank risk cell is diagnosable
The risk cells wrap CDS_MarketValue in IFERROR, which makes "module not imported"
and "the call errored" look identical - both render blank. Nigel is seeing blank
CS01 / IR DV01 / Rec01 with the rest of the sheet working, and there is no way to
tell which from the sheet.

CDS_RiskLoaded() is a zero-argument probe, reported at N20. If it says loaded and
O22:O25 are still blank, the failure is in the call rather than the module, and
the note at N27 says to strip the IFERROR off O22 to surface the real error.

Same pattern as the CDSStrip probe on Steps!B13, which is what made the missing
CDSStrip diagnosable earlier.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/CDS_Pricer.xlsx
+++ b/bloomberg/CDS_Pricer.xlsx
@@ -13703,6 +13703,10 @@
           <t>Protection leg minus premium leg, both to the pricing date.</t>
         </is>
       </c>
+      <c r="N20" s="66">
+        <f>IFERROR(CDS_RiskLoaded(),"CDSRisk.bas NOT imported")</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="67" t="inlineStr">
@@ -13845,6 +13849,11 @@
       <c r="C27" s="65" t="inlineStr">
         <is>
           <t>Market Value / D(T_s) + Accrued Interest. Identically zero when C = S.</t>
+        </is>
+      </c>
+      <c r="N27" s="177" t="inlineStr">
+        <is>
+          <t>If N20 says loaded but O22:O25 are blank, the call itself is failing - not the module. Delete the IFERROR wrapper on O22 to see the real error.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record which quote source the pull uses
Our two-step pull quotes <ticker> & " BEST Curncy", so it is the BEST composite.
CDSW was on CMAN, a single contributor - that alone can explain the gap between
our 66.56 at 5Y and their 51.56, and it is testable by switching the CDSW CDS
Curve dropdown to BEST rather than by guessing at doc clauses.

CDS_Quotes now states the source in a cell instead of leaving it implicit in a
formula string, with the follow-up written down: if BEST still disagrees, the
difference is the instrument rather than the source, and the doc clause behind
the resolved ticker is the thing to check against the XR14 on the deal.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bloomberg/CDS_Pricer.xlsx
+++ b/bloomberg/CDS_Pricer.xlsx
@@ -10303,9 +10303,14 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="65" t="inlineStr">
-        <is>
-          <t>Help Desk H#1330731572. Step 1 BDP(ticker,"CDS_SPREAD_TICKER_nY"); step 2 BDP(returned&amp;" BEST Curncy","PX_LAST"). Tenors 1Y/3Y/5Y/7Y/10Y.</t>
+      <c r="A16" s="67" t="inlineStr">
+        <is>
+          <t>Quote source</t>
+        </is>
+      </c>
+      <c r="B16" s="184" t="inlineStr">
+        <is>
+          <t>BEST, PX_LAST (falls back to PX_MID)</t>
         </is>
       </c>
       <c r="K16" s="139" t="inlineStr">
@@ -10315,9 +10320,9 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="66" t="inlineStr">
-        <is>
-          <t>No Bloomberg export exists for zero-coupon CDS spreads or bootstrapped hazard rates (Help Desk). The credit curve has no external ground truth, unlike the SOFR curve.</t>
+      <c r="A17" s="177" t="inlineStr">
+        <is>
+          <t>Col D resolves the ticker, col F quotes it as &lt;ticker&gt; &amp; " BEST Curncy". That is the BEST composite. CDSW's CDS Curve dropdown must be set to BEST to compare like with like - CMAN, CMAI, CMAL and the rest are single-contributor curves and will not match.</t>
         </is>
       </c>
       <c r="K17" s="139" t="inlineStr">
@@ -10327,9 +10332,9 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="65" t="inlineStr">
-        <is>
-          <t>Bloomberg suggest the credit triangle, hazard = S/(1-R). Exact only for a flat curve. CDSStrip.CDS_StripHazard bootstraps properly; CDS_Validation 13-18 compares the two.</t>
+      <c r="A18" s="177" t="inlineStr">
+        <is>
+          <t>If BEST on CDSW still disagrees, the difference is the instrument, not the source: check the doc clause behind the resolved ticker against the XR14 on the CDSW deal.</t>
         </is>
       </c>
     </row>

</xml_diff>